<commit_message>
feat: Puantaj indirilebilir sablonu gorsel olarak birebir uyumlu olacak sekilde yeniden uretildi (ExcelJS)
</commit_message>
<xml_diff>
--- a/ornek_puantaj_sablonu.xlsx
+++ b/ornek_puantaj_sablonu.xlsx
@@ -1,118 +1,153 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hhasa\OneDrive\Desktop\github\Filo-ERP\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19EC6CD0-01CB-4F43-900E-525C86D1881E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Puantaj" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Puantaj" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="27">
+  <si>
+    <t>Dikkan</t>
+  </si>
+  <si>
+    <t>20.3.2026 CUMA</t>
+  </si>
+  <si>
+    <t>SAAT</t>
+  </si>
+  <si>
+    <t>07:30</t>
+  </si>
+  <si>
+    <t>08:00</t>
+  </si>
+  <si>
+    <t>12:30</t>
+  </si>
+  <si>
+    <t>13:00</t>
+  </si>
+  <si>
+    <t>14:30</t>
+  </si>
+  <si>
+    <t>16:00</t>
+  </si>
+  <si>
+    <t>18:00</t>
+  </si>
+  <si>
+    <t>19:30</t>
+  </si>
+  <si>
+    <t>20:00</t>
+  </si>
+  <si>
+    <t>21:30</t>
+  </si>
+  <si>
+    <t>00:00</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>GÜZERGAH</t>
+  </si>
+  <si>
+    <t>CİNSİ</t>
+  </si>
+  <si>
+    <t>GİRİŞ</t>
+  </si>
+  <si>
+    <t>ÇIKIŞ</t>
+  </si>
+  <si>
+    <t>MURADİYE</t>
+  </si>
+  <si>
+    <t>16+1</t>
+  </si>
+  <si>
+    <t>45 AAB 885</t>
+  </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>16 Mart 2026 Pazartesi</t>
-  </si>
-  <si>
-    <t>NO</t>
-  </si>
-  <si>
-    <t>GÜZERGAH</t>
-  </si>
-  <si>
-    <t>CİNSİ</t>
-  </si>
-  <si>
-    <t>07:30</t>
-  </si>
-  <si>
-    <t>08:00</t>
-  </si>
-  <si>
-    <t>18:00</t>
-  </si>
-  <si>
-    <t>20:30</t>
-  </si>
-  <si>
-    <t>GİRİŞ</t>
-  </si>
-  <si>
-    <t>ÇIKIŞ</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>KARABAĞLAR</t>
-  </si>
-  <si>
-    <t>16+1</t>
-  </si>
-  <si>
-    <t>34ABC123</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>BORNOVA</t>
-  </si>
-  <si>
-    <t>35DEF456</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>BUCA</t>
+    <t>45 AAB 886</t>
+  </si>
+  <si>
+    <t>35 BLT 103</t>
+  </si>
+  <si>
+    <t>LALELİ</t>
   </si>
   <si>
     <t>27+1</t>
-  </si>
-  <si>
-    <t>35XYZ789</t>
-  </si>
-  <si>
-    <t>Dikkan</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFF0000"/>
+    </font>
+    <font>
+      <i/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -120,18 +155,83 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFEEEEEE"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFEEEEEE"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFEEEEEE"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFEEEEEE"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE0E0E0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE0E0E0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE0E0E0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFE0E0E0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -464,149 +564,347 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:N15"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="5.625" customWidth="1"/>
-    <col min="2" max="2" width="20.875" customWidth="1"/>
-    <col min="3" max="3" width="10.875" customWidth="1"/>
-    <col min="4" max="7" width="15.875" customWidth="1"/>
+    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="8" customWidth="1"/>
+    <col min="4" max="14" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="N2" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="N3" s="7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="8">
+        <v>1</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="G4" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="8">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B5" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" s="9">
         <v>3</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10"/>
+      <c r="J6" s="10"/>
+      <c r="K6" s="10"/>
+      <c r="L6" s="10"/>
+      <c r="M6" s="10"/>
+      <c r="N6" s="10"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" s="9">
         <v>4</v>
       </c>
-      <c r="D2" t="s">
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="10"/>
+      <c r="J7" s="10"/>
+      <c r="K7" s="10"/>
+      <c r="L7" s="10"/>
+      <c r="M7" s="10"/>
+      <c r="N7" s="10"/>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" s="9">
         <v>5</v>
       </c>
-      <c r="E2" t="s">
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="10"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="10"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" s="9">
         <v>6</v>
       </c>
-      <c r="F2" t="s">
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
+      <c r="J9" s="10"/>
+      <c r="K9" s="10"/>
+      <c r="L9" s="10"/>
+      <c r="M9" s="10"/>
+      <c r="N9" s="10"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" s="9">
         <v>7</v>
       </c>
-      <c r="G2" t="s">
+      <c r="B10" s="10"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="10"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="10"/>
+      <c r="L10" s="10"/>
+      <c r="M10" s="10"/>
+      <c r="N10" s="10"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" s="9">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" t="s">
-        <v>0</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="10"/>
+      <c r="J11" s="10"/>
+      <c r="K11" s="10"/>
+      <c r="L11" s="10"/>
+      <c r="M11" s="10"/>
+      <c r="N11" s="10"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" s="9">
         <v>9</v>
       </c>
-      <c r="E3" t="s">
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="10"/>
+      <c r="I12" s="10"/>
+      <c r="J12" s="10"/>
+      <c r="K12" s="10"/>
+      <c r="L12" s="10"/>
+      <c r="M12" s="10"/>
+      <c r="N12" s="10"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" s="9">
         <v>10</v>
       </c>
-      <c r="F3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="10"/>
+      <c r="J13" s="10"/>
+      <c r="K13" s="10"/>
+      <c r="L13" s="10"/>
+      <c r="M13" s="10"/>
+      <c r="N13" s="10"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14" s="9">
         <v>11</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="10"/>
+      <c r="I14" s="10"/>
+      <c r="J14" s="10"/>
+      <c r="K14" s="10"/>
+      <c r="L14" s="10"/>
+      <c r="M14" s="10"/>
+      <c r="N14" s="10"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15" s="9">
         <v>12</v>
       </c>
-      <c r="C4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" t="s">
-        <v>0</v>
-      </c>
-      <c r="G4" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E5" t="s">
-        <v>17</v>
-      </c>
-      <c r="F5" t="s">
-        <v>0</v>
-      </c>
-      <c r="G5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D6" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" t="s">
-        <v>0</v>
-      </c>
-      <c r="F6" t="s">
-        <v>21</v>
-      </c>
-      <c r="G6" t="s">
-        <v>0</v>
-      </c>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="10"/>
+      <c r="L15" s="10"/>
+      <c r="M15" s="10"/>
+      <c r="N15" s="10"/>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="D1:N1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A2:C6 D1:G6 B1:C1" numberStoredAsText="1"/>
-  </ignoredErrors>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>